<commit_message>
findings about TDD structure and layering
</commit_message>
<xml_diff>
--- a/Test_Data/analysis/data_v2/fig_tdd_tradeoff.xlsx
+++ b/Test_Data/analysis/data_v2/fig_tdd_tradeoff.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Thesis\thesis\Test_Data\analysis\data_v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8420CC9-6811-49BF-8E66-F56FC81C6A84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B121A09-8150-4182-A327-E3934A2397AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1811,7 +1811,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -1897,12 +1897,7 @@
   <c:spPr>
     <a:noFill/>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
+      <a:noFill/>
       <a:round/>
     </a:ln>
     <a:effectLst/>
@@ -3574,15 +3569,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>23813</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>4762</xdr:rowOff>
+      <xdr:rowOff>10715</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>304800</xdr:colOff>
+      <xdr:colOff>328613</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>80962</xdr:rowOff>
+      <xdr:rowOff>86915</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>